<commit_message>
Lesson 16 - Database - 02.03.2025 - update mo hinh vat ly
</commit_message>
<xml_diff>
--- a/Java23 VoAnhTuan Database Design.xlsx
+++ b/Java23 VoAnhTuan Database Design.xlsx
@@ -8,17 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Hoc Lap Trinh web\java23\3.Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9BCA560-EFEB-4AD9-98DF-5457DE485A24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80FC9608-4773-46C2-9A00-F61EB1411EE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2783" yWindow="2783" windowWidth="17425" windowHeight="8955" tabRatio="588" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-109" yWindow="-109" windowWidth="23452" windowHeight="12561" tabRatio="588" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="B1. Mô hình quan niệm" sheetId="1" r:id="rId1"/>
     <sheet name="B2. Mô hình logic" sheetId="5" r:id="rId2"/>
     <sheet name="ERD - Mô hình logic" sheetId="2" r:id="rId3"/>
     <sheet name="B3. Mô hình quan hệ" sheetId="6" r:id="rId4"/>
-    <sheet name="RD - Mô hình quan hệ" sheetId="3" r:id="rId5"/>
-    <sheet name="DB - Mô hình vật lý" sheetId="4" r:id="rId6"/>
+    <sheet name="B4. Mô hình vật lý" sheetId="7" r:id="rId5"/>
+    <sheet name="RD - Mô hình quan hệ" sheetId="3" r:id="rId6"/>
+    <sheet name="DB - Mô hình vật lý" sheetId="4" r:id="rId7"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -43,7 +44,7 @@
             <sz val="8"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>ADMIN:</t>
         </r>
@@ -52,7 +53,7 @@
             <sz val="8"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 Giá bán được xác định thông qua MatHang và KichCo</t>
@@ -67,7 +68,7 @@
             <sz val="8"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>ADMIN:</t>
         </r>
@@ -76,7 +77,7 @@
             <sz val="8"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 Lưu trữ cùng với KichCo, ChatLieu và MauSac</t>
@@ -87,8 +88,122 @@
 </comments>
 </file>
 
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={D2762586-1568-4CA1-84B1-25C4A6B7BF3D}</author>
+    <author>tc={5BB71AC4-9659-4B49-AE00-20328F749FE8}</author>
+    <author>tc={B0B8351A-F8B3-4EDE-8A43-27DE73070A70}</author>
+    <author>tc={F97C4A89-C3BD-42B8-81A3-F88B0C7B2B49}</author>
+    <author>tc={6B85BF31-59E0-4C41-93B2-A52F1794EB43}</author>
+    <author>tc={757E2222-AC3E-4A43-98F1-5381EF486FA8}</author>
+  </authors>
+  <commentList>
+    <comment ref="K6" authorId="0" shapeId="0" xr:uid="{89E57403-7A0C-47C1-8B87-FEA66CB9DF4C}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Khách
+Nhân Viên
+Quản Lý 
+Giám Đốc</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L6" authorId="1" shapeId="0" xr:uid="{E7ECC064-FD1B-483E-974E-58A73859F84A}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Comment:
+    Chờ xử lý
+Đã xử lý, chờ đóng gói
+Đang đóng gói
+Đang giao hàng
+Giao hàng thành công
+Giao hàng thất bại
+Hủy đơn hàng</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N6" authorId="2" shapeId="0" xr:uid="{835DEFA4-9F05-472C-B196-00B1221F7310}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t xml:space="preserve">Comment:
+    Thanh toán khi nhận hàng
+Thanh toán online - chuyển khoản
+Thanh toán online - thẻ ghi nợ
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Q7" authorId="3" shapeId="0" xr:uid="{ACB75BDC-36D4-43EF-A852-F8A3E1E821A5}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Số lượng bán của mặt hàng trong đơn hàng</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D10" authorId="4" shapeId="0" xr:uid="{ED15A117-9935-478C-B499-3146CE204134}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Số lượng tồn kho theo mặt hàng, kích cỡ</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G12" authorId="5" shapeId="0" xr:uid="{8C29A821-1AB8-4A55-949A-E89C624B8B46}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Comment:
+    Người tạo</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="855" uniqueCount="417">
   <si>
     <t>MatHang</t>
   </si>
@@ -1074,12 +1189,418 @@
   <si>
     <t>đơn vị kích cỡ</t>
   </si>
+  <si>
+    <t>T01_ITEM</t>
+  </si>
+  <si>
+    <t>T02_SIZE</t>
+  </si>
+  <si>
+    <t>T03_ITEM_DETAIL</t>
+  </si>
+  <si>
+    <t>T04_ITEM_GROUP</t>
+  </si>
+  <si>
+    <t>T05_GALLERY</t>
+  </si>
+  <si>
+    <t>T06_ORDER</t>
+  </si>
+  <si>
+    <t>T07_CUSTOMER</t>
+  </si>
+  <si>
+    <t>T08_EMPLOYEE</t>
+  </si>
+  <si>
+    <t>T09_ACCOUNT</t>
+  </si>
+  <si>
+    <t>T10_ROLE</t>
+  </si>
+  <si>
+    <t>T11_ORDER_STATUS</t>
+  </si>
+  <si>
+    <t>T12_ORDER_STATUS_DETAIL</t>
+  </si>
+  <si>
+    <t>T13_PAYMENT_METHOD</t>
+  </si>
+  <si>
+    <t>T14_TITLE</t>
+  </si>
+  <si>
+    <t>T15_BILL</t>
+  </si>
+  <si>
+    <t>T16_ITEM_DETAIL</t>
+  </si>
+  <si>
+    <t>T17_ITEM_RECEIVED_NOTE</t>
+  </si>
+  <si>
+    <t>T18_ITEM_RECEIVED_NOTE_DETAIL</t>
+  </si>
+  <si>
+    <t>T19_PROVIDER</t>
+  </si>
+  <si>
+    <t>C01_ITEM_ID</t>
+  </si>
+  <si>
+    <t>C02_SIZE_ID</t>
+  </si>
+  <si>
+    <t>C03_ITEM_DETAIL_ID</t>
+  </si>
+  <si>
+    <t>C04_ITEM_GROUP_ID</t>
+  </si>
+  <si>
+    <t>C05_ITEM_ID</t>
+  </si>
+  <si>
+    <t>C06_ORDER_ID</t>
+  </si>
+  <si>
+    <t>C07_CUSTOMER_ID</t>
+  </si>
+  <si>
+    <t>C08_EMPLOYEE_ID</t>
+  </si>
+  <si>
+    <t>C09_ACCOUNT_ID</t>
+  </si>
+  <si>
+    <t>C10_ROLE_ID</t>
+  </si>
+  <si>
+    <t>C11_ORDER_STATUS_ID</t>
+  </si>
+  <si>
+    <t>C12_ORDER_ID</t>
+  </si>
+  <si>
+    <t>C13_PAYMENT_METHOD_ID</t>
+  </si>
+  <si>
+    <t>C14_TITLE_ID</t>
+  </si>
+  <si>
+    <t>C15_BILL_ID</t>
+  </si>
+  <si>
+    <t>C16_ORDER_ID</t>
+  </si>
+  <si>
+    <t>C17_IRN_ID</t>
+  </si>
+  <si>
+    <t>C18_IRN_ID</t>
+  </si>
+  <si>
+    <t>C19_PROVIDER_ID</t>
+  </si>
+  <si>
+    <t>C01_ITEM_NAME</t>
+  </si>
+  <si>
+    <t>C02_SIZE_NAME</t>
+  </si>
+  <si>
+    <t>C03_ITEM_ID</t>
+  </si>
+  <si>
+    <t>C04_ITEM_GROUP_NAME</t>
+  </si>
+  <si>
+    <t>C05_COLOR</t>
+  </si>
+  <si>
+    <t>C06_RECEIVER_NAME</t>
+  </si>
+  <si>
+    <t>C07_CUSTOMER_NAME</t>
+  </si>
+  <si>
+    <t>C08_EMPLOYEE_NAME</t>
+  </si>
+  <si>
+    <t>C09_USERNAME</t>
+  </si>
+  <si>
+    <t>C10_ROLE_NAME</t>
+  </si>
+  <si>
+    <t>C11_ORDER_STATUS_DESC</t>
+  </si>
+  <si>
+    <t>C12_ORDER_STATUS_ID</t>
+  </si>
+  <si>
+    <t>C13_PAYMENT_METHOD_NAME</t>
+  </si>
+  <si>
+    <t>C14_TITLE_NAME</t>
+  </si>
+  <si>
+    <t>C15_DELIVERY_FEE</t>
+  </si>
+  <si>
+    <t>C16_ITEM_DETAIL_ID</t>
+  </si>
+  <si>
+    <t>C17_IRN_TIME</t>
+  </si>
+  <si>
+    <t>C18_ITEM_ID</t>
+  </si>
+  <si>
+    <t>C19_PROVIDER_NAME</t>
+  </si>
+  <si>
+    <t>C01_ITEM_GROUP_ID</t>
+  </si>
+  <si>
+    <t>C02_GENDER</t>
+  </si>
+  <si>
+    <t>C03_SIZE_ID</t>
+  </si>
+  <si>
+    <t>C05_IMAGE</t>
+  </si>
+  <si>
+    <t>C06_RECEIVER_PHONE</t>
+  </si>
+  <si>
+    <t>C07_CUSTOMER_PHONE</t>
+  </si>
+  <si>
+    <t>C08_EMPLOYEE_PHONE</t>
+  </si>
+  <si>
+    <t>C09_PASSWORD</t>
+  </si>
+  <si>
+    <t>C12_EMPLOYEE_ID</t>
+  </si>
+  <si>
+    <t>C15_TOTAL_OF_MONEY</t>
+  </si>
+  <si>
+    <t>C16_AMOUNT</t>
+  </si>
+  <si>
+    <t>C17_EMPLOYEE_ID</t>
+  </si>
+  <si>
+    <t>C18_AMOUNT</t>
+  </si>
+  <si>
+    <t>C19_PROVIDER_TAX</t>
+  </si>
+  <si>
+    <t>C02_SIZE_DESC</t>
+  </si>
+  <si>
+    <t>C03_COLOR</t>
+  </si>
+  <si>
+    <t>C06_DELIVERY_ADDRESS</t>
+  </si>
+  <si>
+    <t>C07_CUSTOMER_EMAIL</t>
+  </si>
+  <si>
+    <t>C08_EMPLOYEE_EMAIL</t>
+  </si>
+  <si>
+    <t>C09_ACCOUNT_STATUS</t>
+  </si>
+  <si>
+    <t>C12_LAST_UPDATED</t>
+  </si>
+  <si>
+    <t>C15_ORDER_ID</t>
+  </si>
+  <si>
+    <t>C18_BUY_PRICE</t>
+  </si>
+  <si>
+    <t>C03_SALES_PRICE</t>
+  </si>
+  <si>
+    <t>C06_CUSTOMER_ID</t>
+  </si>
+  <si>
+    <t>C07_CUSTOMER_GENDER</t>
+  </si>
+  <si>
+    <t>C08_EMPLOYEE_GENDER</t>
+  </si>
+  <si>
+    <t>C09_ROLE_ID</t>
+  </si>
+  <si>
+    <t>C18_PROVIDER_ID</t>
+  </si>
+  <si>
+    <t>C03_AMOUNT</t>
+  </si>
+  <si>
+    <t>C06_ORDER_TIME</t>
+  </si>
+  <si>
+    <t>C07_CUSTOMER_DOB</t>
+  </si>
+  <si>
+    <t>C08_EMPLOYEE_DOB</t>
+  </si>
+  <si>
+    <t>C06_PAYMENT_METHOD_ID</t>
+  </si>
+  <si>
+    <t>C07_CUSTOMER_ADDRESS</t>
+  </si>
+  <si>
+    <t>C08_TITLE_ID</t>
+  </si>
+  <si>
+    <t>C06_EMPLOYEE_ID</t>
+  </si>
+  <si>
+    <t>C07_ACCOUNT_ID</t>
+  </si>
+  <si>
+    <t>C08_ACCOUNT_ID</t>
+  </si>
+  <si>
+    <t>Khóa chính này có 2 columns, được tham chiếu từ table khác</t>
+  </si>
+  <si>
+    <t>Bảng tham chiếu sẽ cần có 2 columns này</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Xử lý:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Tạo column mới làm khóa chính đại diện cho table</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">         : Thêm ràng buộc unique cho 2 columns pk cũ</t>
+  </si>
+  <si>
+    <t>1. Database</t>
+  </si>
+  <si>
+    <t>UNIQUE</t>
+  </si>
+  <si>
+    <t>Tìm những đơn hàng bị hủy</t>
+  </si>
+  <si>
+    <t>2. Tables</t>
+  </si>
+  <si>
+    <t>3. Columns</t>
+  </si>
+  <si>
+    <t>Áo sơ mi</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>Size S - Nu - Từ 40 đến 50kg</t>
+  </si>
+  <si>
+    <t>4. Constraints: Primary, Foreign Keys, Unique, NOT NULL, IN SET</t>
+  </si>
+  <si>
+    <t>Quần jean</t>
+  </si>
+  <si>
+    <t>-- View, Function, Procedure, Index, Trigger, Partition</t>
+  </si>
+  <si>
+    <t>XL</t>
+  </si>
+  <si>
+    <t>XXL</t>
+  </si>
+  <si>
+    <t>white</t>
+  </si>
+  <si>
+    <t>file://img01</t>
+  </si>
+  <si>
+    <t>Size S - Nam - Từ 45 đến 55kg</t>
+  </si>
+  <si>
+    <t>file://img03</t>
+  </si>
+  <si>
+    <t>C12_EMPLOYE_ID</t>
+  </si>
+  <si>
+    <t>black</t>
+  </si>
+  <si>
+    <t>file://img02</t>
+  </si>
+  <si>
+    <t>Chờ xử lý</t>
+  </si>
+  <si>
+    <t>NV1</t>
+  </si>
+  <si>
+    <t>--</t>
+  </si>
+  <si>
+    <t>Đang giao</t>
+  </si>
+  <si>
+    <t>NV2</t>
+  </si>
+  <si>
+    <t>T03_ITEM_DETAIL kết hợp của ITEM và SIZE</t>
+  </si>
+  <si>
+    <t>NV4</t>
+  </si>
+  <si>
+    <t>NV6</t>
+  </si>
+  <si>
+    <t>Giao thành công</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1196,17 +1717,54 @@
       <sz val="8"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="8"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
-      <charset val="1"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color theme="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF7030A0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1273,6 +1831,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -1322,7 +1886,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1469,6 +2033,13 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
@@ -1486,20 +2057,44 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2227,7 +2822,7 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:14" ht="43.6" x14ac:dyDescent="0.3">
-      <c r="F3" s="63" t="s">
+      <c r="F3" s="57" t="s">
         <v>271</v>
       </c>
     </row>
@@ -2923,12 +3518,12 @@
       <c r="Q13" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="R13" s="57" t="s">
+      <c r="R13" s="60" t="s">
         <v>68</v>
       </c>
-      <c r="S13" s="57"/>
-      <c r="T13" s="57"/>
-      <c r="U13" s="57"/>
+      <c r="S13" s="60"/>
+      <c r="T13" s="60"/>
+      <c r="U13" s="60"/>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.3">
       <c r="D14" s="5"/>
@@ -2941,10 +3536,10 @@
       <c r="Q14" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="R14" s="57"/>
-      <c r="S14" s="57"/>
-      <c r="T14" s="57"/>
-      <c r="U14" s="57"/>
+      <c r="R14" s="60"/>
+      <c r="S14" s="60"/>
+      <c r="T14" s="60"/>
+      <c r="U14" s="60"/>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
@@ -3261,7 +3856,7 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:14" ht="43.6" x14ac:dyDescent="0.3">
-      <c r="F3" s="63" t="s">
+      <c r="F3" s="57" t="s">
         <v>271</v>
       </c>
     </row>
@@ -3664,13 +4259,11 @@
       <c r="N20" s="2"/>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A23" s="64"/>
-      <c r="C23" s="67" t="s">
+      <c r="C23" s="58" t="s">
         <v>272</v>
       </c>
     </row>
     <row r="24" spans="1:14" s="18" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="65"/>
       <c r="B24"/>
       <c r="C24" s="24" t="s">
         <v>273</v>
@@ -3682,34 +4275,28 @@
       <c r="H24"/>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A25" s="64"/>
       <c r="C25" s="24" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A26" s="64"/>
-    </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A27" s="64"/>
-      <c r="C27" s="67" t="s">
+      <c r="C27" s="58" t="s">
         <v>275</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A28" s="66"/>
+      <c r="A28" s="56"/>
       <c r="C28" s="24" t="s">
         <v>276</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A29" s="64"/>
       <c r="C29" s="24" t="s">
         <v>277</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="C31" s="67" t="s">
+      <c r="C31" s="58" t="s">
         <v>278</v>
       </c>
     </row>
@@ -3724,7 +4311,7 @@
       </c>
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="C35" s="67" t="s">
+      <c r="C35" s="58" t="s">
         <v>281</v>
       </c>
     </row>
@@ -3743,7 +4330,7 @@
     </row>
     <row r="39" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B39" s="49"/>
-      <c r="C39" s="68" t="s">
+      <c r="C39" s="59" t="s">
         <v>284</v>
       </c>
       <c r="D39" s="49"/>
@@ -3772,6 +4359,1089 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9629BCD5-9CC4-4AFD-9A6B-CC273F110309}">
+  <dimension ref="B4:T47"/>
+  <sheetFormatPr defaultRowHeight="14.55" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.21875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="22.77734375" customWidth="1"/>
+    <col min="12" max="12" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="25.109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="28.21875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="31.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="19.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B4" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="Q4" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="R4" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="S4" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="T4" s="1" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="5" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B5" s="67" t="s">
+        <v>307</v>
+      </c>
+      <c r="C5" s="67" t="s">
+        <v>308</v>
+      </c>
+      <c r="D5" s="67" t="s">
+        <v>309</v>
+      </c>
+      <c r="E5" s="67" t="s">
+        <v>310</v>
+      </c>
+      <c r="F5" s="67" t="s">
+        <v>311</v>
+      </c>
+      <c r="G5" s="67" t="s">
+        <v>312</v>
+      </c>
+      <c r="H5" s="66" t="s">
+        <v>313</v>
+      </c>
+      <c r="I5" s="67" t="s">
+        <v>314</v>
+      </c>
+      <c r="J5" s="67" t="s">
+        <v>315</v>
+      </c>
+      <c r="K5" s="67" t="s">
+        <v>316</v>
+      </c>
+      <c r="L5" s="67" t="s">
+        <v>317</v>
+      </c>
+      <c r="M5" s="67" t="s">
+        <v>318</v>
+      </c>
+      <c r="N5" s="67" t="s">
+        <v>319</v>
+      </c>
+      <c r="O5" s="67" t="s">
+        <v>320</v>
+      </c>
+      <c r="P5" s="67" t="s">
+        <v>321</v>
+      </c>
+      <c r="Q5" s="67" t="s">
+        <v>322</v>
+      </c>
+      <c r="R5" s="67" t="s">
+        <v>323</v>
+      </c>
+      <c r="S5" s="67" t="s">
+        <v>324</v>
+      </c>
+      <c r="T5" s="66" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="6" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B6" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="C6" s="68" t="s">
+        <v>327</v>
+      </c>
+      <c r="D6" s="68" t="s">
+        <v>328</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="F6" s="67" t="s">
+        <v>330</v>
+      </c>
+      <c r="G6" s="29" t="s">
+        <v>331</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="M6" s="67" t="s">
+        <v>337</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="O6" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="P6" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="Q6" s="67" t="s">
+        <v>341</v>
+      </c>
+      <c r="R6" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="S6" s="67" t="s">
+        <v>343</v>
+      </c>
+      <c r="T6" s="2" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="7" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B7" s="69" t="s">
+        <v>345</v>
+      </c>
+      <c r="C7" s="68" t="s">
+        <v>346</v>
+      </c>
+      <c r="D7" s="68" t="s">
+        <v>347</v>
+      </c>
+      <c r="E7" s="2"/>
+      <c r="F7" s="67" t="s">
+        <v>348</v>
+      </c>
+      <c r="G7" s="29" t="s">
+        <v>349</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="K7" s="16"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="N7" s="70"/>
+      <c r="O7" s="2"/>
+      <c r="P7" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="Q7" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="R7" s="69" t="s">
+        <v>356</v>
+      </c>
+      <c r="S7" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="T7" s="2" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="8" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B8" s="2"/>
+      <c r="C8" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="D8" s="68" t="s">
+        <v>360</v>
+      </c>
+      <c r="E8" s="16"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="29" t="s">
+        <v>361</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="K8" s="2"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="N8" s="70"/>
+      <c r="O8" s="2"/>
+      <c r="P8" s="69" t="s">
+        <v>366</v>
+      </c>
+      <c r="Q8" s="2"/>
+      <c r="R8" s="2"/>
+      <c r="S8" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="T8" s="2"/>
+    </row>
+    <row r="9" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B9" s="69"/>
+      <c r="C9" s="70"/>
+      <c r="D9" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="E9" s="2"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="69" t="s">
+        <v>369</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="K9" s="2"/>
+      <c r="L9" s="2"/>
+      <c r="M9" s="2"/>
+      <c r="N9" s="70"/>
+      <c r="O9" s="2"/>
+      <c r="P9" s="2"/>
+      <c r="Q9" s="2"/>
+      <c r="R9" s="2"/>
+      <c r="S9" s="69" t="s">
+        <v>373</v>
+      </c>
+      <c r="T9" s="2"/>
+    </row>
+    <row r="10" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B10" s="54"/>
+      <c r="C10" s="70"/>
+      <c r="D10" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
+      <c r="M10" s="2"/>
+      <c r="N10" s="70"/>
+      <c r="O10" s="2"/>
+      <c r="P10" s="2"/>
+      <c r="Q10" s="2"/>
+      <c r="R10" s="2"/>
+      <c r="S10" s="2"/>
+      <c r="T10" s="2"/>
+    </row>
+    <row r="11" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B11" s="54"/>
+      <c r="C11" s="70"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="54" t="s">
+        <v>378</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="I11" s="69" t="s">
+        <v>380</v>
+      </c>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
+      <c r="L11" s="2"/>
+      <c r="M11" s="2"/>
+      <c r="N11" s="70"/>
+      <c r="O11" s="69"/>
+      <c r="P11" s="69"/>
+      <c r="Q11" s="69"/>
+      <c r="R11" s="69"/>
+      <c r="S11" s="69"/>
+      <c r="T11" s="69"/>
+    </row>
+    <row r="12" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B12" s="70"/>
+      <c r="C12" s="70"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="54" t="s">
+        <v>381</v>
+      </c>
+      <c r="H12" s="69" t="s">
+        <v>382</v>
+      </c>
+      <c r="I12" s="69" t="s">
+        <v>383</v>
+      </c>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
+      <c r="L12" s="2"/>
+      <c r="M12" s="2"/>
+      <c r="N12" s="70"/>
+      <c r="O12" s="69"/>
+      <c r="P12" s="69"/>
+      <c r="Q12" s="69"/>
+      <c r="R12" s="69"/>
+      <c r="S12" s="69"/>
+      <c r="T12" s="69"/>
+    </row>
+    <row r="13" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B13" s="70"/>
+      <c r="C13" s="70"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="16"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
+      <c r="L13" s="2"/>
+      <c r="M13" s="2"/>
+      <c r="N13" s="70"/>
+      <c r="O13" s="2"/>
+      <c r="P13" s="2"/>
+      <c r="Q13" s="2"/>
+      <c r="R13" s="2"/>
+      <c r="S13" s="2"/>
+      <c r="T13" s="2"/>
+    </row>
+    <row r="14" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B14" s="70"/>
+      <c r="C14" s="70"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="54"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
+      <c r="L14" s="2"/>
+      <c r="M14" s="2"/>
+      <c r="N14" s="70"/>
+      <c r="O14" s="2"/>
+      <c r="P14" s="2"/>
+      <c r="Q14" s="2"/>
+      <c r="R14" s="2"/>
+      <c r="S14" s="2"/>
+      <c r="T14" s="2"/>
+    </row>
+    <row r="15" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B15" s="70"/>
+      <c r="C15" s="70"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
+      <c r="L15" s="2"/>
+      <c r="M15" s="2"/>
+      <c r="N15" s="70"/>
+      <c r="O15" s="2"/>
+      <c r="P15" s="2"/>
+      <c r="Q15" s="2"/>
+      <c r="R15" s="2"/>
+      <c r="S15" s="2"/>
+      <c r="T15" s="2"/>
+    </row>
+    <row r="16" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B16" s="70"/>
+      <c r="C16" s="70"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
+      <c r="L16" s="2"/>
+      <c r="M16" s="2"/>
+      <c r="N16" s="70"/>
+      <c r="O16" s="2"/>
+      <c r="P16" s="2"/>
+      <c r="Q16" s="2"/>
+      <c r="R16" s="2"/>
+      <c r="S16" s="2"/>
+      <c r="T16" s="2"/>
+    </row>
+    <row r="17" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B17" s="70"/>
+      <c r="C17" s="70"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2"/>
+      <c r="K17" s="2"/>
+      <c r="L17" s="2"/>
+      <c r="M17" s="2"/>
+      <c r="N17" s="70"/>
+      <c r="O17" s="2"/>
+      <c r="P17" s="2"/>
+      <c r="Q17" s="2"/>
+      <c r="R17" s="2"/>
+      <c r="S17" s="2"/>
+      <c r="T17" s="2"/>
+    </row>
+    <row r="18" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B18" s="70"/>
+      <c r="C18" s="70"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
+      <c r="L18" s="2"/>
+      <c r="M18" s="2"/>
+      <c r="N18" s="70"/>
+      <c r="O18" s="2"/>
+      <c r="P18" s="2"/>
+      <c r="Q18" s="2"/>
+      <c r="R18" s="2"/>
+      <c r="S18" s="2"/>
+      <c r="T18" s="2"/>
+    </row>
+    <row r="19" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B19" s="70"/>
+      <c r="C19" s="70"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
+      <c r="K19" s="2"/>
+      <c r="L19" s="2"/>
+      <c r="M19" s="2"/>
+      <c r="N19" s="70"/>
+      <c r="O19" s="2"/>
+      <c r="P19" s="2"/>
+      <c r="Q19" s="2"/>
+      <c r="R19" s="2"/>
+      <c r="S19" s="2"/>
+      <c r="T19" s="2"/>
+    </row>
+    <row r="20" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B20" s="70"/>
+      <c r="C20" s="70"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2"/>
+      <c r="K20" s="2"/>
+      <c r="L20" s="2"/>
+      <c r="M20" s="2"/>
+      <c r="N20" s="70"/>
+      <c r="O20" s="2"/>
+      <c r="P20" s="2"/>
+      <c r="Q20" s="2"/>
+      <c r="R20" s="2"/>
+      <c r="S20" s="2"/>
+      <c r="T20" s="2"/>
+    </row>
+    <row r="21" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="I21" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="22" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="I22" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="23" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="I23" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="24" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="I24" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="25" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B25" t="s">
+        <v>388</v>
+      </c>
+      <c r="F25" s="23" t="s">
+        <v>288</v>
+      </c>
+      <c r="I25" s="23" t="s">
+        <v>289</v>
+      </c>
+      <c r="J25" s="71" t="s">
+        <v>389</v>
+      </c>
+      <c r="K25" s="71"/>
+      <c r="N25" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="26" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B26" t="s">
+        <v>391</v>
+      </c>
+      <c r="F26" s="23" t="s">
+        <v>307</v>
+      </c>
+      <c r="G26" s="23" t="s">
+        <v>326</v>
+      </c>
+      <c r="I26" s="23" t="s">
+        <v>308</v>
+      </c>
+      <c r="J26" t="s">
+        <v>327</v>
+      </c>
+      <c r="K26" t="s">
+        <v>346</v>
+      </c>
+      <c r="L26" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="27" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B27" t="s">
+        <v>392</v>
+      </c>
+      <c r="F27" s="23">
+        <v>1</v>
+      </c>
+      <c r="G27" s="23" t="s">
+        <v>393</v>
+      </c>
+      <c r="H27" s="23"/>
+      <c r="I27" s="23">
+        <v>1</v>
+      </c>
+      <c r="J27" s="23" t="s">
+        <v>394</v>
+      </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
+      <c r="L27" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="28" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B28" t="s">
+        <v>396</v>
+      </c>
+      <c r="F28" s="23">
+        <v>2</v>
+      </c>
+      <c r="G28" s="23" t="s">
+        <v>397</v>
+      </c>
+      <c r="H28" s="23"/>
+      <c r="I28" s="23">
+        <v>2</v>
+      </c>
+      <c r="J28" s="23" t="s">
+        <v>85</v>
+      </c>
+      <c r="K28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B29" s="24" t="s">
+        <v>398</v>
+      </c>
+      <c r="F29" s="23"/>
+      <c r="G29" s="23"/>
+      <c r="H29" s="23"/>
+      <c r="I29" s="23">
+        <v>3</v>
+      </c>
+      <c r="J29" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="K29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="F30" t="s">
+        <v>292</v>
+      </c>
+      <c r="I30" s="23">
+        <v>4</v>
+      </c>
+      <c r="J30" s="23" t="s">
+        <v>399</v>
+      </c>
+      <c r="K30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="F31" s="23" t="s">
+        <v>311</v>
+      </c>
+      <c r="G31" s="23" t="s">
+        <v>330</v>
+      </c>
+      <c r="H31" s="23" t="s">
+        <v>348</v>
+      </c>
+      <c r="I31" s="23">
+        <v>5</v>
+      </c>
+      <c r="J31" s="23" t="s">
+        <v>400</v>
+      </c>
+      <c r="K31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="F32" s="23">
+        <v>1</v>
+      </c>
+      <c r="G32" s="23" t="s">
+        <v>401</v>
+      </c>
+      <c r="H32" s="72" t="s">
+        <v>402</v>
+      </c>
+      <c r="I32" s="23">
+        <v>6</v>
+      </c>
+      <c r="J32" s="23" t="s">
+        <v>394</v>
+      </c>
+      <c r="K32">
+        <v>1</v>
+      </c>
+      <c r="L32" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="33" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B33" s="73" t="s">
+        <v>299</v>
+      </c>
+      <c r="C33" s="74"/>
+      <c r="D33" s="74"/>
+      <c r="E33" s="74"/>
+      <c r="F33" s="23">
+        <v>1</v>
+      </c>
+      <c r="G33" s="23" t="s">
+        <v>401</v>
+      </c>
+      <c r="H33" s="72" t="s">
+        <v>404</v>
+      </c>
+      <c r="I33" s="23">
+        <v>7</v>
+      </c>
+      <c r="J33" s="23" t="s">
+        <v>85</v>
+      </c>
+      <c r="K33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B34" s="73" t="s">
+        <v>318</v>
+      </c>
+      <c r="C34" s="73" t="s">
+        <v>337</v>
+      </c>
+      <c r="D34" s="73" t="s">
+        <v>405</v>
+      </c>
+      <c r="E34" s="73" t="s">
+        <v>365</v>
+      </c>
+      <c r="F34" s="23">
+        <v>1</v>
+      </c>
+      <c r="G34" s="23" t="s">
+        <v>406</v>
+      </c>
+      <c r="H34" s="72" t="s">
+        <v>407</v>
+      </c>
+      <c r="I34" s="23">
+        <v>8</v>
+      </c>
+      <c r="J34" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="K34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B35" s="75">
+        <v>1</v>
+      </c>
+      <c r="C35" s="75" t="s">
+        <v>408</v>
+      </c>
+      <c r="D35" s="75" t="s">
+        <v>409</v>
+      </c>
+      <c r="E35" s="76" t="s">
+        <v>410</v>
+      </c>
+      <c r="I35" s="23">
+        <v>9</v>
+      </c>
+      <c r="J35" s="23" t="s">
+        <v>399</v>
+      </c>
+      <c r="K35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B36" s="75">
+        <v>1</v>
+      </c>
+      <c r="C36" s="75" t="s">
+        <v>100</v>
+      </c>
+      <c r="D36" s="75" t="s">
+        <v>409</v>
+      </c>
+      <c r="E36" s="76" t="s">
+        <v>410</v>
+      </c>
+      <c r="I36" s="23">
+        <v>10</v>
+      </c>
+      <c r="J36" s="23" t="s">
+        <v>400</v>
+      </c>
+      <c r="K36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B37" s="75">
+        <v>1</v>
+      </c>
+      <c r="C37" s="75" t="s">
+        <v>411</v>
+      </c>
+      <c r="D37" s="75" t="s">
+        <v>412</v>
+      </c>
+      <c r="E37" s="75"/>
+      <c r="H37" s="23"/>
+      <c r="J37" s="77" t="s">
+        <v>400</v>
+      </c>
+      <c r="K37" s="35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B38" s="75">
+        <v>2</v>
+      </c>
+      <c r="C38" s="75" t="s">
+        <v>408</v>
+      </c>
+      <c r="D38" s="75" t="s">
+        <v>412</v>
+      </c>
+      <c r="E38" s="76" t="s">
+        <v>410</v>
+      </c>
+      <c r="F38" s="23" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="39" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B39" s="75">
+        <v>2</v>
+      </c>
+      <c r="C39" s="75" t="s">
+        <v>100</v>
+      </c>
+      <c r="D39" s="75" t="s">
+        <v>414</v>
+      </c>
+      <c r="E39" s="76" t="s">
+        <v>410</v>
+      </c>
+      <c r="F39" s="23" t="s">
+        <v>328</v>
+      </c>
+      <c r="G39" s="23" t="s">
+        <v>347</v>
+      </c>
+      <c r="H39" s="23" t="s">
+        <v>360</v>
+      </c>
+      <c r="I39" s="23" t="s">
+        <v>368</v>
+      </c>
+      <c r="J39" s="23" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="40" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B40" s="75">
+        <v>2</v>
+      </c>
+      <c r="C40" s="75" t="s">
+        <v>411</v>
+      </c>
+      <c r="D40" s="75" t="s">
+        <v>415</v>
+      </c>
+      <c r="E40" s="75"/>
+      <c r="F40" s="23">
+        <v>1</v>
+      </c>
+      <c r="G40" s="23">
+        <v>1</v>
+      </c>
+      <c r="H40" s="23" t="s">
+        <v>401</v>
+      </c>
+      <c r="I40" s="23">
+        <v>220</v>
+      </c>
+      <c r="J40" s="23">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="41" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B41" s="75">
+        <v>2</v>
+      </c>
+      <c r="C41" s="75" t="s">
+        <v>416</v>
+      </c>
+      <c r="D41" s="75" t="s">
+        <v>415</v>
+      </c>
+      <c r="E41" s="75"/>
+      <c r="F41" s="23">
+        <v>1</v>
+      </c>
+      <c r="G41" s="23">
+        <v>1</v>
+      </c>
+      <c r="H41" s="23" t="s">
+        <v>406</v>
+      </c>
+      <c r="I41" s="23">
+        <v>230</v>
+      </c>
+      <c r="J41" s="23">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="42" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B42" s="75"/>
+      <c r="C42" s="75"/>
+      <c r="D42" s="75"/>
+      <c r="E42" s="75"/>
+      <c r="F42" s="23">
+        <v>1</v>
+      </c>
+      <c r="G42" s="23">
+        <v>2</v>
+      </c>
+      <c r="H42" s="23"/>
+      <c r="I42" s="23">
+        <v>200</v>
+      </c>
+      <c r="J42" s="23">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="43" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B43" s="78"/>
+      <c r="C43" s="78"/>
+      <c r="D43" s="78"/>
+      <c r="E43" s="78"/>
+      <c r="F43" s="23">
+        <v>1</v>
+      </c>
+      <c r="G43" s="23">
+        <v>3</v>
+      </c>
+      <c r="H43" s="23"/>
+      <c r="I43" s="23"/>
+      <c r="J43" s="23">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="44" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B44" s="79"/>
+      <c r="C44" s="79"/>
+      <c r="D44" s="79"/>
+      <c r="E44" s="79"/>
+      <c r="F44" s="23">
+        <v>1</v>
+      </c>
+      <c r="G44" s="23">
+        <v>5</v>
+      </c>
+      <c r="H44" s="23"/>
+      <c r="I44" s="23"/>
+      <c r="J44" s="23">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="45" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="F45" s="23">
+        <v>2</v>
+      </c>
+      <c r="G45" s="23">
+        <v>6</v>
+      </c>
+      <c r="H45" s="23"/>
+      <c r="I45" s="23"/>
+      <c r="J45" s="23">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="46" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="F46" s="23">
+        <v>2</v>
+      </c>
+      <c r="G46" s="23">
+        <v>9</v>
+      </c>
+      <c r="H46" s="23"/>
+      <c r="I46" s="23"/>
+      <c r="J46" s="23">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="47" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="F47" s="23">
+        <v>2</v>
+      </c>
+      <c r="G47" s="23">
+        <v>10</v>
+      </c>
+      <c r="H47" s="23"/>
+      <c r="I47" s="23"/>
+      <c r="J47" s="23">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="J25:K25"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="H32" r:id="rId1" xr:uid="{188DEF51-13F8-4C40-B45A-54E0B8183F3C}"/>
+    <hyperlink ref="H33" r:id="rId2" display="file://img01" xr:uid="{FDFDFA17-57CE-4797-A312-90E2A6F92B04}"/>
+    <hyperlink ref="H34" r:id="rId3" display="file://img01" xr:uid="{95BFC119-EDF9-466C-86BD-09B315841648}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId4"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A2:AJ77"/>
   <sheetFormatPr defaultRowHeight="14.55" x14ac:dyDescent="0.3"/>
@@ -4047,10 +5717,10 @@
       <c r="W18" s="5"/>
     </row>
     <row r="19" spans="3:35" x14ac:dyDescent="0.3">
-      <c r="P19" s="62" t="s">
+      <c r="P19" s="65" t="s">
         <v>11</v>
       </c>
-      <c r="Q19" s="62"/>
+      <c r="Q19" s="65"/>
       <c r="T19" s="4" t="s">
         <v>9</v>
       </c>
@@ -4068,10 +5738,10 @@
       <c r="P20" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="Q20" s="61" t="s">
+      <c r="Q20" s="64" t="s">
         <v>14</v>
       </c>
-      <c r="R20" s="61"/>
+      <c r="R20" s="64"/>
       <c r="T20" s="4" t="s">
         <v>94</v>
       </c>
@@ -4089,10 +5759,10 @@
       <c r="P21" s="4">
         <v>1</v>
       </c>
-      <c r="Q21" s="61" t="s">
+      <c r="Q21" s="64" t="s">
         <v>99</v>
       </c>
-      <c r="R21" s="61"/>
+      <c r="R21" s="64"/>
       <c r="T21" s="4" t="s">
         <v>94</v>
       </c>
@@ -4110,10 +5780,10 @@
       <c r="P22" s="4">
         <v>2</v>
       </c>
-      <c r="Q22" s="61" t="s">
+      <c r="Q22" s="64" t="s">
         <v>100</v>
       </c>
-      <c r="R22" s="61"/>
+      <c r="R22" s="64"/>
       <c r="T22" s="4" t="s">
         <v>94</v>
       </c>
@@ -4131,10 +5801,10 @@
       <c r="P23" s="4">
         <v>3</v>
       </c>
-      <c r="Q23" s="61" t="s">
+      <c r="Q23" s="64" t="s">
         <v>101</v>
       </c>
-      <c r="R23" s="61"/>
+      <c r="R23" s="64"/>
       <c r="T23" s="4"/>
       <c r="U23" s="4"/>
       <c r="V23" s="4"/>
@@ -4153,10 +5823,10 @@
       <c r="P24" s="4">
         <v>4</v>
       </c>
-      <c r="Q24" s="61" t="s">
+      <c r="Q24" s="64" t="s">
         <v>102</v>
       </c>
-      <c r="R24" s="61"/>
+      <c r="R24" s="64"/>
       <c r="T24" s="4" t="s">
         <v>95</v>
       </c>
@@ -4801,16 +6471,16 @@
       </c>
     </row>
     <row r="48" spans="3:36" x14ac:dyDescent="0.3">
-      <c r="C48" s="58" t="s">
+      <c r="C48" s="61" t="s">
         <v>221</v>
       </c>
-      <c r="D48" s="59"/>
-      <c r="E48" s="59"/>
-      <c r="F48" s="59"/>
-      <c r="G48" s="59"/>
-      <c r="H48" s="59"/>
-      <c r="I48" s="59"/>
-      <c r="J48" s="59"/>
+      <c r="D48" s="62"/>
+      <c r="E48" s="62"/>
+      <c r="F48" s="62"/>
+      <c r="G48" s="62"/>
+      <c r="H48" s="62"/>
+      <c r="I48" s="62"/>
+      <c r="J48" s="62"/>
       <c r="O48" s="29">
         <v>3</v>
       </c>
@@ -4840,16 +6510,16 @@
       </c>
     </row>
     <row r="49" spans="3:32" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C49" s="60" t="s">
+      <c r="C49" s="63" t="s">
         <v>220</v>
       </c>
-      <c r="D49" s="60"/>
-      <c r="E49" s="60"/>
-      <c r="F49" s="60"/>
-      <c r="G49" s="60"/>
-      <c r="H49" s="60"/>
-      <c r="I49" s="60"/>
-      <c r="J49" s="60"/>
+      <c r="D49" s="63"/>
+      <c r="E49" s="63"/>
+      <c r="F49" s="63"/>
+      <c r="G49" s="63"/>
+      <c r="H49" s="63"/>
+      <c r="I49" s="63"/>
+      <c r="J49" s="63"/>
       <c r="O49" s="29">
         <v>4</v>
       </c>
@@ -5304,7 +6974,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="B2:N26"/>
   <sheetFormatPr defaultRowHeight="14.55" x14ac:dyDescent="0.3"/>

</xml_diff>